<commit_message>
autosave 2026-08-20 12:53 · 2 file(s)
</commit_message>
<xml_diff>
--- a/KOBRA-S1-STARTUP-BOM.xlsx
+++ b/KOBRA-S1-STARTUP-BOM.xlsx
@@ -423,19 +423,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J22"/>
+  <dimension ref="A1:K25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="34" customWidth="1" min="3" max="3"/>
-    <col width="58" customWidth="1" min="4" max="4"/>
-    <col width="5" customWidth="1" min="5" max="5"/>
-    <col width="10" customWidth="1" min="6" max="6"/>
-    <col width="10" customWidth="1" min="7" max="7"/>
-    <col width="26" customWidth="1" min="8" max="8"/>
-    <col width="22" customWidth="1" min="9" max="9"/>
-    <col width="52" customWidth="1" min="10" max="10"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="52" customWidth="1" min="4" max="4"/>
+    <col width="44" customWidth="1" min="5" max="5"/>
+    <col width="5" customWidth="1" min="6" max="6"/>
+    <col width="9" customWidth="1" min="7" max="7"/>
+    <col width="9" customWidth="1" min="8" max="8"/>
+    <col width="24" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
+    <col width="48" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -461,30 +462,35 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
+          <t>Color</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
           <t>Qty</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Est $ each</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Est $ line</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Vendor examples</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Feed path</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
@@ -513,16 +519,21 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
           <t>owned</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr"/>
       <c r="I2" t="inlineStr"/>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>Quick-release hotend cartridges ONLY - generic MK8/V6 nozzles do NOT fit</t>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>Quick-release hotend cartridges ONLY - generic MK8/V6 nozzles do NOT fit. Color doctrine: black + gray + OD green accent, nothing else.</t>
         </is>
       </c>
     </row>
@@ -539,42 +550,47 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>PLA - calibration/iteration</t>
+          <t>PLA - calibration</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>1.75mm, +/-0.02mm tolerance, 1kg PLASTIC spool (no cardboard in ACE), regular gloss finish - NO matte (ACE false-tangle), NO silk. Black or gray.</t>
+          <t>1.75mm, +/-0.02mm, 1kg PLASTIC spool, regular gloss - NO matte (ACE false-tangle), NO silk</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>LIGHT GRAY - calibration standard: max defect/layer-line visibility</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
           <t>14</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>28</t>
-        </is>
-      </c>
       <c r="H3" t="inlineStr">
         <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
           <t>Elegoo / Sunlu / Anycubic</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr">
+      <c r="J3" t="inlineStr">
         <is>
           <t>ACE Pro</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>Calibration cubes, tolerance tests, shape drafts. Never ships.</t>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>Tuning spool. Gray shows what white blows out and black hides.</t>
         </is>
       </c>
     </row>
@@ -591,42 +607,47 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>PETG - v1 enclosure material</t>
+          <t>PLA - shape drafts</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>1.75mm, +/-0.03mm, 1kg plastic spool. 2x black + 1x production color candidate.</t>
+          <t>same spec as above</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>BLACK - previews product look</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>51</t>
+          <t>14</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Overture / Polymaker PolyLite</t>
+          <t>14</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
+          <t>Elegoo / Sunlu / Anycubic</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
           <t>ACE Pro</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>Dry 6-8h @ 55C in ACE before first run - new spools are never dry</t>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>Iteration drafts in product color. Never ships.</t>
         </is>
       </c>
     </row>
@@ -638,47 +659,52 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Adhesion</t>
+          <t>Filament</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Glue stick 2-pack</t>
+          <t>PETG - v1 production</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Plain PVP stick, 22g (disappearing purple fine)</t>
+          <t>1.75mm, +/-0.03mm, 1kg plastic spool</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>BLACK - production primary (hides seams/layers, photographs clean)</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>2</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>17</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>Elmer's</t>
+          <t>34</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Overture / Polymaker PolyLite</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>RELEASE layer for PETG (bonds too hard to PEI); adhesion aid for ASA later</t>
+          <t>ACE Pro</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>Dry 6-8h @ 55C in ACE before first run. SlimeVR is IMU-based - black has zero tracking penalty.</t>
         </is>
       </c>
     </row>
@@ -690,47 +716,52 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Plate prep</t>
+          <t>Filament</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>IPA 91%+ 1qt + microfiber cloths 6pk</t>
+          <t>PETG - palette accent</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>91% or higher isopropyl</t>
+          <t>same spec</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>OD / ARMY GREEN - on-palette accent candidate</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>17</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>any pharmacy</t>
+          <t>17</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Polymaker PolyLite</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>Degrease plate between prints. Skip if stocked.</t>
+          <t>ACE Pro</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>One production color + one accent = product line. Rainbow = hobbyist.</t>
         </is>
       </c>
     </row>
@@ -742,47 +773,52 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Storage</t>
+          <t>Adhesion</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Vacuum filament storage kit</t>
+          <t>Glue stick 2-pack</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>~10 bags w/ one-way valves + hand pump + rechargeable silica gel + mini hygrometers</t>
+          <t>Plain PVP stick, 22g (disappearing purple fine)</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>28</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>28</t>
+          <t>4</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>SUNLU kit or generic</t>
+          <t>4</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Elmer's</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>Tallahassee humidity = enemy #1. Every spool not in the ACE lives sealed.</t>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>RELEASE layer for PETG (bonds too hard to PEI); adhesion aid for ASA later</t>
         </is>
       </c>
     </row>
@@ -794,151 +830,166 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Spares</t>
+          <t>Plate prep</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Spare 0.4mm hotend unit</t>
+          <t>IPA 91%+ 1qt + microfiber 6pk</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Anycubic Kobra S1 official quick-release cartridge, brass 0.4mm</t>
+          <t>91% or higher isopropyl</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>8</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>Anycubic store</t>
+          <t>8</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>any pharmacy</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>60-second clog recovery mid-run. Buy official only.</t>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>Degrease plate between prints. Skip if stocked.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Filament</t>
+          <t>Storage</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>ASA - production enclosures</t>
+          <t>Vacuum filament storage kit</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>1.75mm, 1kg plastic spool, black (OD/army green optional for palette)</t>
+          <t>~10 bags w/ valves + hand pump + rechargeable silica + mini hygrometers</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>46</t>
+          <t>28</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>Polymaker PolyLite ASA</t>
+          <t>28</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>ACE Pro (dry separately first)</t>
+          <t>SUNLU or generic</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>95C heat resist, UV stable, satin finish. Dry @ 70C in S2 BEFORE loading - ALWAYS in FL. Ventilate room during runs.</t>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>FL humidity = enemy #1. Every spool not in the ACE lives sealed.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Drying</t>
+          <t>Spares</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Standalone filament dryer</t>
+          <t>Spare 0.4mm hotend unit</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Single-spool, reaches 70C (ACE maxes at 55C - cannot dry ASA)</t>
+          <t>Anycubic Kobra S1 official quick-release cartridge, brass 0.4mm</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>45</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>45</t>
+          <t>18</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>Sunlu FilaDryer S2</t>
+          <t>18</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Anycubic store</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>Upgrade path: S4 quad if throughput demands</t>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>60-second clog recovery. Official only.</t>
         </is>
       </c>
     </row>
@@ -950,47 +1001,52 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Hardware</t>
+          <t>Filament</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Heat-set insert kit M3</t>
+          <t>ASA - production primary</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Brass knurled inserts, ~5.0mm OD x 4.0mm length (std 3D-print spec), 100+ pcs</t>
+          <t>1.75mm, 1kg plastic spool</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>BLACK - carbon-black pigment = most dimensionally consistent + most UV-proven</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>23</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>ruthex / CNC Kitchen style</t>
+          <t>23</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Polymaker PolyLite ASA</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>Threads into printed bosses; the pro answer for enclosures that open</t>
+          <t>ACE Pro (dry separately)</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>Dry @ 70C in S2 BEFORE loading, always. Ventilate during runs. 95C heat resist, satin premium finish.</t>
         </is>
       </c>
     </row>
@@ -1002,47 +1058,52 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Tools</t>
+          <t>Filament</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>M3 heat-set installation tips</t>
+          <t>ASA - palette accent</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Tip set fitting standard soldering iron</t>
+          <t>same spec</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>OD / ARMY GREEN</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>23</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>ruthex / generic</t>
+          <t>23</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Polymaker PolyLite ASA</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>Assumes iron owned; add basic 60W adjustable +$20 if not</t>
+          <t>ACE Pro (dry separately)</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>Second production colorway once black is dialed</t>
         </is>
       </c>
     </row>
@@ -1054,47 +1115,52 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Hardware</t>
+          <t>Drying</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>M3 screw assortment</t>
+          <t>Standalone filament dryer</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Socket-head + button-head, 6/8/10/12/16/20mm + nuts + washers, black-oxide or stainless</t>
+          <t>Single-spool, reaches 70C (ACE maxes at 55C)</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>45</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>any assortment box</t>
+          <t>45</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Sunlu FilaDryer S2</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>Button-head on visible exterior faces</t>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>Covers ASA/CF drying the ACE cannot. Upgrade path: S4 quad.</t>
         </is>
       </c>
     </row>
@@ -1106,47 +1172,52 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Spares</t>
+          <t>Hardware</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>0.6mm hotend unit</t>
+          <t>Heat-set insert kit M3</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Anycubic official quick-release, brass 0.6mm</t>
+          <t>Brass knurled, ~5.0mm OD x 4.0mm length, 100+ pcs</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>brass</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>18</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>Anycubic store</t>
+          <t>18</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>ruthex / CNC Kitchen style</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>Draft iterations ~40% faster; keep 0.4 for final surfaces</t>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>Threads into printed bosses</t>
         </is>
       </c>
     </row>
@@ -1158,47 +1229,52 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Maintenance</t>
+          <t>Tools</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Super Lube 21030</t>
+          <t>M3 heat-set installation tips</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Synthetic grease w/ PTFE, 3oz tube</t>
+          <t>Tip set for standard soldering iron</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>Super Lube</t>
+          <t>12</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>ruthex / generic</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>Rails + lead screws every 1-2 months heavy use</t>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>+$20 basic 60W iron if not owned</t>
         </is>
       </c>
     </row>
@@ -1210,54 +1286,55 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Spares</t>
+          <t>Hardware</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>PTFE tube + cutter + couplings</t>
+          <t>M3 screw assortment</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>2m tube 1.9mm ID x 4.0mm OD (Capricorn-class) + tube cutter + PC4-M6 quick couplings 4pk</t>
+          <t>Socket + button head, 6/8/10/12/16/20mm + nuts/washers</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>BLACK-OXIDE - matches black enclosures; button-head on visible faces</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>18</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>Capricorn / generic</t>
+          <t>18</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>assortment box</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>ACE feed paths are wear items; couplings = known community fix</t>
-        </is>
-      </c>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1267,146 +1344,161 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Hardened-steel 0.4mm hotend</t>
+          <t>0.6mm hotend unit</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Anycubic official all-metal hardened quick-release</t>
+          <t>Anycubic official quick-release, brass 0.6mm</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>28</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>28</t>
+          <t>20</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
           <t>Anycubic store</t>
         </is>
       </c>
-      <c r="I17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>REQUIRED before any carbon-fiber filament touches the machine</t>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>Drafts ~40% faster; 0.4 for final surfaces</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Filament</t>
+          <t>Maintenance</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>PETG-CF - premium tier</t>
+          <t>Super Lube 21030</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>1.75mm, 1kg</t>
+          <t>Synthetic PTFE grease, 3oz</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>28</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>28</t>
+          <t>10</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>Polymaker / eSun</t>
+          <t>10</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>DIRECT FEED ONLY</t>
+          <t>Super Lube</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>Never through ACE (wears channels). Hardened hotend only. Dry @ 70C.</t>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>Rails + lead screws, every 1-2 months heavy use</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Filament</t>
+          <t>Spares</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>TPU 95A - gaskets/soft parts</t>
+          <t>PTFE tube + cutter + couplings</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>1.75mm, 1kg</t>
+          <t>2m tube 1.9mm ID x 4.0mm OD (Capricorn-class) + cutter + PC4-M6 couplings 4pk</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>15</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>Overture / Polymaker</t>
+          <t>15</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>DIRECT FEED ONLY</t>
+          <t>Capricorn / generic</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>Single-color direct only - cannot run through ACE</t>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>ACE feed paths are wear items</t>
         </is>
       </c>
     </row>
@@ -1418,47 +1510,52 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Plates</t>
+          <t>Spares</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Second build plate</t>
+          <t>Hardened-steel 0.4mm hotend</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Official Kobra S1 plate, OPPOSITE finish to shipped one (smooth vs textured PEI)</t>
+          <t>Anycubic official all-metal hardened quick-release</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
           <t>28</t>
         </is>
       </c>
-      <c r="G20" t="inlineStr">
+      <c r="H20" t="inlineStr">
         <is>
           <t>28</t>
         </is>
       </c>
-      <c r="H20" t="inlineStr">
+      <c r="I20" t="inlineStr">
         <is>
           <t>Anycubic store</t>
         </is>
       </c>
-      <c r="I20" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>Two product surface finishes + hot-swap throughput</t>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>REQUIRED before any CF filament</t>
         </is>
       </c>
     </row>
@@ -1470,47 +1567,52 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Safety</t>
+          <t>Filament</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Smart plug + smoke detector</t>
+          <t>PETG-CF - premium tier</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Kasa-class wifi plug + basic detector near printer</t>
+          <t>1.75mm, 1kg</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>BLACK - CF is inherently black, no choice exists; dead-matte</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>28</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>TP-Link Kasa</t>
+          <t>28</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Polymaker / eSun</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>Remote kill + fire sense for unattended production runs</t>
+          <t>DIRECT FEED ONLY</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>Never through ACE. Hardened hotend only. Dry @ 70C.</t>
         </is>
       </c>
     </row>
@@ -1522,47 +1624,223 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
+          <t>Filament</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>TPU 95A - gaskets/soft parts</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>1.75mm, 1kg</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>BLACK - wear parts hide service grime</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>22</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>22</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>Overture / Polymaker</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>DIRECT FEED ONLY</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>Cannot run through ACE</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Plates</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Second build plate</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Official Kobra S1, OPPOSITE finish to shipped (smooth vs textured PEI)</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>Anycubic store</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>Textured face-down = uniform premium bottom surface</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Safety</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Smart plug + smoke detector</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Kasa-class wifi plug + detector near printer</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>TP-Link Kasa</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>Remote kill + fire sense for unattended runs</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
           <t>Air</t>
         </is>
       </c>
-      <c r="C22" t="inlineStr">
+      <c r="C25" t="inlineStr">
         <is>
           <t>Carbon filter (BentoBox style)</t>
         </is>
       </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>Activated carbon pellets ~$10 + printable box (free)</t>
-        </is>
-      </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="F22" t="inlineStr">
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Activated carbon pellets + printable box (free, print in black PETG)</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
         <is>
           <t>10</t>
         </is>
       </c>
-      <c r="G22" t="inlineStr">
+      <c r="H25" t="inlineStr">
         <is>
           <t>10</t>
         </is>
       </c>
-      <c r="H22" t="inlineStr">
+      <c r="I25" t="inlineStr">
         <is>
           <t>print it</t>
         </is>
       </c>
-      <c r="I22" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J22" t="inlineStr">
-        <is>
-          <t>Scrubs ASA styrene smell in-chamber; still ventilate</t>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>Scrubs ASA styrene; still ventilate</t>
         </is>
       </c>
     </row>

</xml_diff>